<commit_message>
Separated the cluster analyses into their own folder within both Zinc and Copper folders
</commit_message>
<xml_diff>
--- a/Zinc/6. Statistical data analysis/Multiple linear regression/MLR.xlsx
+++ b/Zinc/6. Statistical data analysis/Multiple linear regression/MLR.xlsx
@@ -6,13 +6,15 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Final_Table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Full_Model_Coefficients" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Full_Model_Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">Predictor</t>
   </si>
@@ -60,6 +62,42 @@
   </si>
   <si>
     <t xml:space="preserve">log_SO4_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Std. Error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pr(&gt;|t|)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Intercept)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Residual standard error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R-squared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjusted R-squared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-statistic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numerator df</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denominator df</t>
   </si>
 </sst>
 </file>
@@ -596,4 +634,303 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-0.0000000000000000617781055114893</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.0125495419681964</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.00000000000000492273787107531</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.999999999999996</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.926129393360342</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0155685705205599</v>
+      </c>
+      <c r="D3" t="n">
+        <v>59.4871181099956</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000407445292713326</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.045902911120325</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0137915474323035</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-3.32833652972168</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.000968206680282881</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.171555958972215</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0151480361796393</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11.3252937171358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.000000000000000000000000174427624549752</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.433480863024706</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0195327863536029</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-22.1924744978715</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.00000000000000000000000000000000000000000000000000000000000000000002348995250765</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-0.0306781682211757</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0366870030113996</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.836213528034526</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.403615260024787</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-0.105116944474928</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.040792112005142</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-2.5768938970769</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0103853856747688</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-0.388232447015612</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0379593457391267</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-10.2275853141336</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.00000000000000000000129760820114478</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-0.00434951235588958</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0270789781729081</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.160623208457739</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.872484456559793</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.0286183582210191</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0253418361627276</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.12929300139311</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.259561121620467</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.0788965001548262</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0551794495247269</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.42981673130812</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.153677191547443</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-0.0542583840178608</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0284125917325186</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-1.9096597919915</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.0570085786456517</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.236784284287834</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.945670483756954</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.943933202714298</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="n">
+        <v>544.339378913288</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="n">
+        <v>344</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>